<commit_message>
auto: atualiza dados 06/2026
</commit_message>
<xml_diff>
--- a/Faturamento_ClickImpresso.xlsx
+++ b/Faturamento_ClickImpresso.xlsx
@@ -534,13 +534,13 @@
         <v>6</v>
       </c>
       <c r="G2" t="n">
-        <v>338</v>
+        <v>467</v>
       </c>
       <c r="H2" t="n">
-        <v>25019.9</v>
+        <v>33190.04</v>
       </c>
       <c r="I2" t="n">
-        <v>-58</v>
+        <v>-60</v>
       </c>
     </row>
     <row r="3">
@@ -2496,13 +2496,13 @@
         <v>6</v>
       </c>
       <c r="G56" t="n">
-        <v>300</v>
+        <v>436</v>
       </c>
       <c r="H56" t="n">
-        <v>18001.2</v>
+        <v>25790.08</v>
       </c>
       <c r="I56" t="n">
-        <v>-75</v>
+        <v>-63</v>
       </c>
     </row>
     <row r="57">
@@ -3866,13 +3866,13 @@
         <v>6</v>
       </c>
       <c r="G94" t="n">
-        <v>212</v>
+        <v>285</v>
       </c>
       <c r="H94" t="n">
-        <v>15719.5</v>
+        <v>22071.4</v>
       </c>
       <c r="I94" t="n">
-        <v>-81</v>
+        <v>-65</v>
       </c>
     </row>
     <row r="95">
@@ -5976,13 +5976,13 @@
         <v>6</v>
       </c>
       <c r="G152" t="n">
-        <v>147</v>
+        <v>217</v>
       </c>
       <c r="H152" t="n">
-        <v>13511.8</v>
+        <v>15736.2</v>
       </c>
       <c r="I152" t="n">
-        <v>-71</v>
+        <v>-59</v>
       </c>
     </row>
     <row r="153">
@@ -6606,13 +6606,13 @@
         <v>6</v>
       </c>
       <c r="G170" t="n">
-        <v>124</v>
+        <v>182</v>
       </c>
       <c r="H170" t="n">
-        <v>4972.1</v>
+        <v>12560.2</v>
       </c>
       <c r="I170" t="n">
-        <v>-82</v>
+        <v>-64</v>
       </c>
     </row>
     <row r="171">
@@ -7643,13 +7643,13 @@
         <v>6</v>
       </c>
       <c r="G199" t="n">
-        <v>172</v>
+        <v>237</v>
       </c>
       <c r="H199" t="n">
-        <v>12595.36</v>
+        <v>15342.41</v>
       </c>
       <c r="I199" t="n">
-        <v>-74</v>
+        <v>-61</v>
       </c>
     </row>
     <row r="200">
@@ -9161,10 +9161,10 @@
         <v>6</v>
       </c>
       <c r="G241" t="n">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="H241" t="n">
-        <v>2295.62</v>
+        <v>4030.04</v>
       </c>
     </row>
     <row r="242">
@@ -9229,13 +9229,13 @@
         <v>6</v>
       </c>
       <c r="G243" t="n">
-        <v>263</v>
+        <v>339</v>
       </c>
       <c r="H243" t="n">
-        <v>19535.93</v>
+        <v>44403.03</v>
       </c>
       <c r="I243" t="n">
-        <v>-78</v>
+        <v>-64</v>
       </c>
     </row>
     <row r="244">
@@ -10451,13 +10451,13 @@
         <v>6</v>
       </c>
       <c r="G277" t="n">
-        <v>130</v>
+        <v>181</v>
       </c>
       <c r="H277" t="n">
-        <v>7949.6</v>
+        <v>10502.5</v>
       </c>
       <c r="I277" t="n">
-        <v>-64</v>
+        <v>-63</v>
       </c>
     </row>
     <row r="278">
@@ -11340,13 +11340,13 @@
         <v>6</v>
       </c>
       <c r="G302" t="n">
-        <v>183</v>
+        <v>246</v>
       </c>
       <c r="H302" t="n">
-        <v>7833.6</v>
+        <v>11145.5</v>
       </c>
       <c r="I302" t="n">
-        <v>-82</v>
+        <v>-62</v>
       </c>
     </row>
     <row r="303">
@@ -12858,13 +12858,13 @@
         <v>6</v>
       </c>
       <c r="G344" t="n">
-        <v>385</v>
+        <v>563</v>
       </c>
       <c r="H344" t="n">
-        <v>43875.04</v>
+        <v>57636.8</v>
       </c>
       <c r="I344" t="n">
-        <v>-78</v>
+        <v>-68</v>
       </c>
     </row>
     <row r="345">
@@ -17447,13 +17447,13 @@
         <v>6</v>
       </c>
       <c r="G469" t="n">
-        <v>62</v>
+        <v>106</v>
       </c>
       <c r="H469" t="n">
-        <v>6207.5</v>
+        <v>9539.120000000001</v>
       </c>
       <c r="I469" t="n">
-        <v>-46</v>
+        <v>-21</v>
       </c>
     </row>
     <row r="470">
@@ -17929,13 +17929,13 @@
         <v>6</v>
       </c>
       <c r="G483" t="n">
-        <v>269</v>
+        <v>350</v>
       </c>
       <c r="H483" t="n">
-        <v>12152.32</v>
+        <v>14714.92</v>
       </c>
       <c r="I483" t="n">
-        <v>-63</v>
+        <v>-52</v>
       </c>
     </row>
     <row r="484">
@@ -18720,10 +18720,13 @@
         <v>6</v>
       </c>
       <c r="G506" t="n">
-        <v>157</v>
+        <v>233</v>
       </c>
       <c r="H506" t="n">
-        <v>14140.93</v>
+        <v>26929.54</v>
+      </c>
+      <c r="I506" t="n">
+        <v>-59</v>
       </c>
     </row>
     <row r="507">
@@ -25180,10 +25183,10 @@
         <v>6</v>
       </c>
       <c r="G696" t="n">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="H696" t="n">
-        <v>2517.92</v>
+        <v>4362.72</v>
       </c>
     </row>
     <row r="697">
@@ -25316,13 +25319,13 @@
         <v>6</v>
       </c>
       <c r="G700" t="n">
-        <v>3342</v>
+        <v>4641</v>
       </c>
       <c r="H700" t="n">
-        <v>241780.36</v>
+        <v>352334.84</v>
       </c>
       <c r="I700" t="n">
-        <v>-76</v>
+        <v>-62</v>
       </c>
     </row>
     <row r="701">
@@ -32310,13 +32313,13 @@
         <v>6</v>
       </c>
       <c r="G890" t="n">
-        <v>198</v>
+        <v>260</v>
       </c>
       <c r="H890" t="n">
-        <v>13402.34</v>
+        <v>16958.72</v>
       </c>
       <c r="I890" t="n">
-        <v>-75</v>
+        <v>-64</v>
       </c>
     </row>
     <row r="891">
@@ -34050,13 +34053,13 @@
         <v>6</v>
       </c>
       <c r="G938" t="n">
-        <v>281</v>
+        <v>379</v>
       </c>
       <c r="H938" t="n">
-        <v>21991.2</v>
+        <v>27363.12</v>
       </c>
       <c r="I938" t="n">
-        <v>-76</v>
+        <v>-63</v>
       </c>
     </row>
     <row r="939">

</xml_diff>